<commit_message>
Update 3 terms in bcio_setting.xlsx
</commit_message>
<xml_diff>
--- a/Setting/bcio_setting.xlsx
+++ b/Setting/bcio_setting.xlsx
@@ -445,54 +445,54 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Parent</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'has part' [BFO:0000051]</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'has BCI context' [BCIOR:000004]</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'has attribute' [RO:0000053]</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'comparatively evaluates' [BCIOR:000006]</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'has output' [RO:0002234]</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'realises' [BFO:0000055]</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'has disposition' [RO:0000091]</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'is about' [IAO:0000136]</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>REL 'is attribute of' [RO:0000052]</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'has part' [BFO:0000051]</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'has BCI context' [BCIOR:000004]</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'has attribute' [RO:0000053]</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'comparatively evaluates' [BCIOR:000006]</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'has output' [RO:0002234]</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'realises' [BFO:0000055]</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'has disposition' [RO:0000091]</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'is about' [IAO:0000136]</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Parent</t>
-        </is>
-      </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Synonyms</t>
@@ -505,62 +505,62 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>Logical definition</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Examples</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Cross reference</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Sub-ontology</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>Curator note</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Comment</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Cross reference</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Curator</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Curation status</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Informal definition</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>To be reviewed by</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>BFO entity</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Reviewer query</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Sub-ontology</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Examples</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Informal definition</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>Logical definition</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>BFO entity</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>Curator</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
@@ -590,7 +590,11 @@
           <t>A form of transporation which can transport patients for health treatment, and in some instances will also provide out-of-hospital healthcare to the patient.</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>transportation [BCIO:026041]</t>
+        </is>
+      </c>
       <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="n"/>
       <c r="G2" s="2" t="n"/>
@@ -599,29 +603,25 @@
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>transportation [BCIO:026041]</t>
-        </is>
-      </c>
+      <c r="M2" s="2" t="n"/>
       <c r="N2" s="2" t="n"/>
       <c r="O2" s="2" t="n"/>
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="n"/>
-      <c r="S2" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U2" s="2" t="n"/>
-      <c r="V2" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="n"/>
       <c r="Z2" s="2" t="n"/>
@@ -649,24 +649,24 @@
           <t>A material entity that is a human made strcuture with firm connection between its foundation and the ground.</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>material entity [BFO:0000040]</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>RW</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
@@ -691,7 +691,11 @@
           <t>An attribute of location describing the overall socioeconomic state of a location.</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>attribute of location [BCIO:026003]</t>
+        </is>
+      </c>
       <c r="E4" s="2" t="n"/>
       <c r="F4" s="2" t="n"/>
       <c r="G4" s="2" t="n"/>
@@ -700,31 +704,27 @@
       <c r="J4" s="2" t="n"/>
       <c r="K4" s="2" t="n"/>
       <c r="L4" s="2" t="n"/>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>attribute of location [BCIO:026003]</t>
-        </is>
-      </c>
+      <c r="M4" s="2" t="n"/>
       <c r="N4" s="2" t="n"/>
       <c r="O4" s="2" t="n"/>
       <c r="P4" s="2" t="n"/>
-      <c r="Q4" s="2" t="n"/>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>disadvantaged area; crime rates; World Bank Classifications</t>
+        </is>
+      </c>
       <c r="R4" s="2" t="n"/>
-      <c r="S4" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T4" s="2" t="n"/>
+      <c r="S4" s="2" t="n"/>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U4" s="2" t="n"/>
-      <c r="V4" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V4" s="2" t="n"/>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>disadvantaged area; crime rates; World Bank Classifications</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X4" s="2" t="n"/>
@@ -754,7 +754,11 @@
           <t>A community facility designed to entertain or amuse.</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>community facility [BCIO:026029]</t>
+        </is>
+      </c>
       <c r="E5" s="2" t="n"/>
       <c r="F5" s="2" t="n"/>
       <c r="G5" s="2" t="n"/>
@@ -763,31 +767,27 @@
       <c r="J5" s="2" t="n"/>
       <c r="K5" s="2" t="n"/>
       <c r="L5" s="2" t="n"/>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>community facility [BCIO:026029]</t>
-        </is>
-      </c>
+      <c r="M5" s="2" t="n"/>
       <c r="N5" s="2" t="n"/>
       <c r="O5" s="2" t="n"/>
       <c r="P5" s="2" t="n"/>
-      <c r="Q5" s="2" t="n"/>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>cinema; theatre; disco</t>
+        </is>
+      </c>
       <c r="R5" s="2" t="n"/>
-      <c r="S5" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T5" s="2" t="n"/>
+      <c r="S5" s="2" t="n"/>
+      <c r="T5" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U5" s="2" t="n"/>
-      <c r="V5" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V5" s="2" t="n"/>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>cinema; theatre; disco</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X5" s="2" t="n"/>
@@ -819,7 +819,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention physical setting</t>
+          <t>specifically dependent continuant [BFO:0000020]</t>
         </is>
       </c>
       <c r="E6" s="2" t="n"/>
@@ -832,7 +832,7 @@
       <c r="L6" s="2" t="n"/>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>specifically dependent continuant [BFO:0000020]</t>
+          <t>behaviour change intervention physical setting</t>
         </is>
       </c>
       <c r="N6" s="2" t="n"/>
@@ -840,27 +840,27 @@
       <c r="P6" s="2" t="n"/>
       <c r="Q6" s="2" t="n"/>
       <c r="R6" s="2" t="n"/>
-      <c r="S6" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T6" s="2" t="n"/>
+      <c r="S6" s="2" t="n"/>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U6" s="2" t="n"/>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W6" s="2" t="n"/>
+          <t>JH; BG</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X6" s="2" t="n"/>
       <c r="Y6" s="2" t="n"/>
       <c r="Z6" s="2" t="n"/>
-      <c r="AA6" s="2" t="inlineStr">
-        <is>
-          <t>JH; BG</t>
-        </is>
-      </c>
+      <c r="AA6" s="2" t="n"/>
       <c r="AB6" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -884,7 +884,7 @@
           <t>A landform consisting of loose rock particles such as sand, gravel, shingle, pebbles, cobble, or even shell fragments along the shoreline of a body of wate</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>outdoor environment [BCIO:026046]</t>
         </is>
@@ -899,14 +899,14 @@
           <t>ENVO:00000091</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>Setting</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -931,7 +931,11 @@
           <t>A healthcare facility that is run by a care home organization and is the bearer of a care home function.</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n"/>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>healthcare facility [OMRSE:00000102]</t>
+        </is>
+      </c>
       <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="n"/>
@@ -940,29 +944,25 @@
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="n"/>
       <c r="L8" s="2" t="n"/>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>healthcare facility [OMRSE:00000102]</t>
-        </is>
-      </c>
+      <c r="M8" s="2" t="n"/>
       <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="n"/>
       <c r="P8" s="2" t="n"/>
       <c r="Q8" s="2" t="n"/>
       <c r="R8" s="2" t="n"/>
-      <c r="S8" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T8" s="2" t="n"/>
+      <c r="S8" s="2" t="n"/>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U8" s="2" t="n"/>
-      <c r="V8" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W8" s="2" t="n"/>
+      <c r="V8" s="2" t="n"/>
+      <c r="W8" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X8" s="2" t="n"/>
       <c r="Y8" s="2" t="n"/>
       <c r="Z8" s="2" t="n"/>
@@ -990,7 +990,11 @@
           <t xml:space="preserve">A facility used by a group of people living in the same place or having a particular characteristic in common. </t>
         </is>
       </c>
-      <c r="D9" s="2" t="n"/>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>facility [OMRSE:00000062]</t>
+        </is>
+      </c>
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="n"/>
@@ -999,31 +1003,27 @@
       <c r="J9" s="2" t="n"/>
       <c r="K9" s="2" t="n"/>
       <c r="L9" s="2" t="n"/>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>facility [OMRSE:00000062]</t>
-        </is>
-      </c>
+      <c r="M9" s="2" t="n"/>
       <c r="N9" s="2" t="n"/>
       <c r="O9" s="2" t="n"/>
       <c r="P9" s="2" t="n"/>
-      <c r="Q9" s="2" t="n"/>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>food bank; recycling centre</t>
+        </is>
+      </c>
       <c r="R9" s="2" t="n"/>
-      <c r="S9" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T9" s="2" t="n"/>
+      <c r="S9" s="2" t="n"/>
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U9" s="2" t="n"/>
-      <c r="V9" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V9" s="2" t="n"/>
       <c r="W9" s="2" t="inlineStr">
         <is>
-          <t>food bank; recycling centre</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X9" s="2" t="n"/>
@@ -1053,7 +1053,11 @@
           <t>A clinic providing healthcare services to people in a certain area</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n"/>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>healthcare facility [OMRSE:00000102]</t>
+        </is>
+      </c>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="n"/>
@@ -1062,31 +1066,27 @@
       <c r="J10" s="2" t="n"/>
       <c r="K10" s="2" t="n"/>
       <c r="L10" s="2" t="n"/>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>healthcare facility [OMRSE:00000102]</t>
-        </is>
-      </c>
+      <c r="M10" s="2" t="n"/>
       <c r="N10" s="2" t="n"/>
       <c r="O10" s="2" t="n"/>
       <c r="P10" s="2" t="n"/>
-      <c r="Q10" s="2" t="n"/>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>polyclinic</t>
+        </is>
+      </c>
       <c r="R10" s="2" t="n"/>
-      <c r="S10" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T10" s="2" t="n"/>
+      <c r="S10" s="2" t="n"/>
+      <c r="T10" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U10" s="2" t="n"/>
-      <c r="V10" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V10" s="2" t="n"/>
       <c r="W10" s="2" t="inlineStr">
         <is>
-          <t>polyclinic</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X10" s="2" t="n"/>
@@ -1116,7 +1116,11 @@
           <t>A healthcare facility to treat patients in the community without them staying overnight.</t>
         </is>
       </c>
-      <c r="D11" s="2" t="n"/>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>community healthcare facility [BCIO:026019]</t>
+        </is>
+      </c>
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="n"/>
@@ -1125,29 +1129,25 @@
       <c r="J11" s="2" t="n"/>
       <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="n"/>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>community healthcare facility [BCIO:026019]</t>
-        </is>
-      </c>
+      <c r="M11" s="2" t="n"/>
       <c r="N11" s="2" t="n"/>
       <c r="O11" s="2" t="n"/>
       <c r="P11" s="2" t="n"/>
       <c r="Q11" s="2" t="n"/>
       <c r="R11" s="2" t="n"/>
-      <c r="S11" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T11" s="2" t="n"/>
+      <c r="S11" s="2" t="n"/>
+      <c r="T11" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U11" s="2" t="n"/>
-      <c r="V11" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W11" s="2" t="n"/>
+      <c r="V11" s="2" t="n"/>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X11" s="2" t="n"/>
       <c r="Y11" s="2" t="n"/>
       <c r="Z11" s="2" t="n"/>
@@ -1175,7 +1175,11 @@
           <t>A geographical location of a country where the intervention takes place.</t>
         </is>
       </c>
-      <c r="D12" s="2" t="n"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>geographic location [GAZ:00000448]</t>
+        </is>
+      </c>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="n"/>
       <c r="G12" s="2" t="n"/>
@@ -1184,31 +1188,27 @@
       <c r="J12" s="2" t="n"/>
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="n"/>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>geographic location [GAZ:00000448]</t>
-        </is>
-      </c>
+      <c r="M12" s="2" t="n"/>
       <c r="N12" s="2" t="n"/>
       <c r="O12" s="2" t="n"/>
       <c r="P12" s="2" t="n"/>
-      <c r="Q12" s="2" t="n"/>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom; Spain</t>
+        </is>
+      </c>
       <c r="R12" s="2" t="n"/>
-      <c r="S12" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T12" s="2" t="n"/>
+      <c r="S12" s="2" t="n"/>
+      <c r="T12" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U12" s="2" t="n"/>
-      <c r="V12" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V12" s="2" t="n"/>
       <c r="W12" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom; Spain</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X12" s="2" t="n"/>
@@ -1238,7 +1238,11 @@
           <t>A facility where individuals are being reprimanded, detained or imprisoned.</t>
         </is>
       </c>
-      <c r="D13" s="2" t="n"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>facility [OMRSE:00000062]</t>
+        </is>
+      </c>
       <c r="E13" s="2" t="n"/>
       <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="n"/>
@@ -1247,31 +1251,27 @@
       <c r="J13" s="2" t="n"/>
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="n"/>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>facility [OMRSE:00000062]</t>
-        </is>
-      </c>
+      <c r="M13" s="2" t="n"/>
       <c r="N13" s="2" t="n"/>
       <c r="O13" s="2" t="n"/>
       <c r="P13" s="2" t="n"/>
-      <c r="Q13" s="2" t="n"/>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>prison</t>
+        </is>
+      </c>
       <c r="R13" s="2" t="n"/>
-      <c r="S13" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T13" s="2" t="n"/>
+      <c r="S13" s="2" t="n"/>
+      <c r="T13" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U13" s="2" t="n"/>
-      <c r="V13" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V13" s="2" t="n"/>
       <c r="W13" s="2" t="inlineStr">
         <is>
-          <t>prison</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X13" s="2" t="n"/>
@@ -1301,7 +1301,11 @@
           <t>A healthcare facility where dental healthcare is provided.</t>
         </is>
       </c>
-      <c r="D14" s="2" t="n"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>healthcare facility [OMRSE:00000102]</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="2" t="n"/>
       <c r="G14" s="2" t="n"/>
@@ -1310,29 +1314,25 @@
       <c r="J14" s="2" t="n"/>
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="n"/>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>healthcare facility [OMRSE:00000102]</t>
-        </is>
-      </c>
+      <c r="M14" s="2" t="n"/>
       <c r="N14" s="2" t="n"/>
       <c r="O14" s="2" t="n"/>
       <c r="P14" s="2" t="n"/>
       <c r="Q14" s="2" t="n"/>
       <c r="R14" s="2" t="n"/>
-      <c r="S14" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T14" s="2" t="n"/>
+      <c r="S14" s="2" t="n"/>
+      <c r="T14" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U14" s="2" t="n"/>
-      <c r="V14" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W14" s="2" t="n"/>
+      <c r="V14" s="2" t="n"/>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X14" s="2" t="n"/>
       <c r="Y14" s="2" t="n"/>
       <c r="Z14" s="2" t="n"/>
@@ -1360,7 +1360,11 @@
           <t>A healthcare facility led by doctors.</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>healthcare facility [OMRSE:00000102]</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="n"/>
@@ -1369,41 +1373,37 @@
       <c r="J15" s="2" t="n"/>
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="n"/>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>healthcare facility [OMRSE:00000102]</t>
-        </is>
-      </c>
+      <c r="M15" s="2" t="n"/>
       <c r="N15" s="2" t="n"/>
       <c r="O15" s="2" t="n"/>
       <c r="P15" s="2" t="n"/>
-      <c r="Q15" s="2" t="n"/>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>general practitioners surgery; doctor surgery</t>
+        </is>
+      </c>
       <c r="R15" s="2" t="n"/>
-      <c r="S15" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T15" s="2" t="n"/>
+      <c r="S15" s="2" t="n"/>
+      <c r="T15" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U15" s="2" t="n"/>
       <c r="V15" s="2" t="inlineStr">
         <is>
-          <t>Setting</t>
+          <t>AW</t>
         </is>
       </c>
       <c r="W15" s="2" t="inlineStr">
         <is>
-          <t>general practitioners surgery; doctor surgery</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X15" s="2" t="n"/>
       <c r="Y15" s="2" t="n"/>
       <c r="Z15" s="2" t="n"/>
-      <c r="AA15" s="2" t="inlineStr">
-        <is>
-          <t>AW</t>
-        </is>
-      </c>
+      <c r="AA15" s="2" t="n"/>
       <c r="AB15" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1427,7 +1427,11 @@
           <t>A rehabilitation facility to assist the recovery of people with drug or alcohol addiction.</t>
         </is>
       </c>
-      <c r="D16" s="2" t="n"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>rehabilitation facility [OMRSE:00000106]</t>
+        </is>
+      </c>
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="n"/>
@@ -1436,29 +1440,25 @@
       <c r="J16" s="2" t="n"/>
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="n"/>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>rehabilitation facility [OMRSE:00000106]</t>
-        </is>
-      </c>
+      <c r="M16" s="2" t="n"/>
       <c r="N16" s="2" t="n"/>
       <c r="O16" s="2" t="n"/>
       <c r="P16" s="2" t="n"/>
       <c r="Q16" s="2" t="n"/>
       <c r="R16" s="2" t="n"/>
-      <c r="S16" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T16" s="2" t="n"/>
+      <c r="S16" s="2" t="n"/>
+      <c r="T16" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U16" s="2" t="n"/>
-      <c r="V16" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W16" s="2" t="n"/>
+      <c r="V16" s="2" t="n"/>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X16" s="2" t="n"/>
       <c r="Y16" s="2" t="n"/>
       <c r="Z16" s="2" t="n"/>
@@ -1486,7 +1486,11 @@
           <t>An educational facility in which pre-school education is provided.</t>
         </is>
       </c>
-      <c r="D17" s="2" t="n"/>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>educational facility [BCIO:026022]</t>
+        </is>
+      </c>
       <c r="E17" s="2" t="n"/>
       <c r="F17" s="2" t="n"/>
       <c r="G17" s="2" t="n"/>
@@ -1495,31 +1499,27 @@
       <c r="J17" s="2" t="n"/>
       <c r="K17" s="2" t="n"/>
       <c r="L17" s="2" t="n"/>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>educational facility [BCIO:026022]</t>
-        </is>
-      </c>
+      <c r="M17" s="2" t="n"/>
       <c r="N17" s="2" t="n"/>
       <c r="O17" s="2" t="n"/>
       <c r="P17" s="2" t="n"/>
-      <c r="Q17" s="2" t="n"/>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nursery school </t>
+        </is>
+      </c>
       <c r="R17" s="2" t="n"/>
-      <c r="S17" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T17" s="2" t="n"/>
+      <c r="S17" s="2" t="n"/>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U17" s="2" t="n"/>
-      <c r="V17" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V17" s="2" t="n"/>
       <c r="W17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">nursery school </t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X17" s="2" t="n"/>
@@ -1549,7 +1549,11 @@
           <t>A facility in which formal education is provided to a student population.</t>
         </is>
       </c>
-      <c r="D18" s="2" t="n"/>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>facility [OMRSE:00000062]</t>
+        </is>
+      </c>
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="n"/>
@@ -1558,29 +1562,25 @@
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n"/>
-      <c r="M18" s="2" t="inlineStr">
-        <is>
-          <t>facility [OMRSE:00000062]</t>
-        </is>
-      </c>
+      <c r="M18" s="2" t="n"/>
       <c r="N18" s="2" t="n"/>
       <c r="O18" s="2" t="n"/>
       <c r="P18" s="2" t="n"/>
       <c r="Q18" s="2" t="n"/>
       <c r="R18" s="2" t="n"/>
-      <c r="S18" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T18" s="2" t="n"/>
+      <c r="S18" s="2" t="n"/>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U18" s="2" t="n"/>
-      <c r="V18" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W18" s="2" t="n"/>
+      <c r="V18" s="2" t="n"/>
+      <c r="W18" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X18" s="2" t="n"/>
       <c r="Y18" s="2" t="n"/>
       <c r="Z18" s="2" t="n"/>
@@ -1608,7 +1608,7 @@
           <t>A health care facility that bears a function to provide emergency healthcare services and the acute care of patients who present without prior appointment, having arrived either by their own means or by ambulance</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>hospital facility [OMRSE:00000063]</t>
         </is>
@@ -1623,14 +1623,14 @@
           <t>OMRSE:00000114</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>Setting</t>
         </is>
       </c>
       <c r="AB19" t="inlineStr">
@@ -1655,7 +1655,7 @@
           <t>An architectural structure that bears some function.</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>architectural structure [OMRSE:00000061]</t>
         </is>
@@ -1670,19 +1670,19 @@
           <t>OMRSE:00000062</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr">
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="AA20" t="inlineStr">
-        <is>
-          <t>RW</t>
         </is>
       </c>
       <c r="AB20" t="inlineStr">
@@ -1707,7 +1707,11 @@
           <t>A facility of a building or group of buildings where goods are manufactured or assembled chiefly by machine</t>
         </is>
       </c>
-      <c r="D21" s="2" t="n"/>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>facility [OMRSE:00000062]</t>
+        </is>
+      </c>
       <c r="E21" s="2" t="n"/>
       <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="n"/>
@@ -1716,29 +1720,25 @@
       <c r="J21" s="2" t="n"/>
       <c r="K21" s="2" t="n"/>
       <c r="L21" s="2" t="n"/>
-      <c r="M21" s="2" t="inlineStr">
-        <is>
-          <t>facility [OMRSE:00000062]</t>
-        </is>
-      </c>
+      <c r="M21" s="2" t="n"/>
       <c r="N21" s="2" t="n"/>
       <c r="O21" s="2" t="n"/>
       <c r="P21" s="2" t="n"/>
       <c r="Q21" s="2" t="n"/>
       <c r="R21" s="2" t="n"/>
-      <c r="S21" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T21" s="2" t="n"/>
+      <c r="S21" s="2" t="n"/>
+      <c r="T21" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U21" s="2" t="n"/>
-      <c r="V21" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W21" s="2" t="n"/>
+      <c r="V21" s="2" t="n"/>
+      <c r="W21" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X21" s="2" t="n"/>
       <c r="Y21" s="2" t="n"/>
       <c r="Z21" s="2" t="n"/>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>forest area</t>
+          <t>forested area</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1766,7 +1766,7 @@
           <t>An area with a high density of trees. A small forest may be called a wood</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>outdoor environment [BCIO:026046]</t>
         </is>
@@ -1781,19 +1781,19 @@
           <t>ENVO:00000111</t>
         </is>
       </c>
-      <c r="S22" t="inlineStr">
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="AA22" t="inlineStr">
-        <is>
-          <t>RW</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -1818,7 +1818,7 @@
           <t>A reference to a place on the Earth, by its name or by its geographical location</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>spatial region [BFO:0000006]</t>
         </is>
@@ -1833,19 +1833,19 @@
           <t>GAZ:00000448</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr">
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>lz</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="AA23" t="inlineStr">
-        <is>
-          <t>lz</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -1870,7 +1870,7 @@
           <t>An area in which grasses (Graminae) are a significant component of the vegetation</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>outdoor environment [BCIO:026046]</t>
         </is>
@@ -1885,19 +1885,19 @@
           <t>ENVO:00000106</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr">
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="AA24" t="inlineStr">
-        <is>
-          <t>RW</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
@@ -1922,7 +1922,7 @@
           <t>A facility that’s administered by a health care organisation for the purpose of providing health care to a patient population</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>facility [OMRSE:00000062]</t>
         </is>
@@ -1937,19 +1937,19 @@
           <t>OMRSE:00000102</t>
         </is>
       </c>
-      <c r="S25" t="inlineStr">
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="AA25" t="inlineStr">
-        <is>
-          <t>RW</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -1974,7 +1974,11 @@
           <t>An area social and economic condition described to have a high-income, whether at a country or within-country level.</t>
         </is>
       </c>
-      <c r="D26" s="2" t="n"/>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>area social and economic condition [BCIO:026004]</t>
+        </is>
+      </c>
       <c r="E26" s="2" t="n"/>
       <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="n"/>
@@ -1983,31 +1987,27 @@
       <c r="J26" s="2" t="n"/>
       <c r="K26" s="2" t="n"/>
       <c r="L26" s="2" t="n"/>
-      <c r="M26" s="2" t="inlineStr">
-        <is>
-          <t>area social and economic condition [BCIO:026004]</t>
-        </is>
-      </c>
+      <c r="M26" s="2" t="n"/>
       <c r="N26" s="2" t="n"/>
       <c r="O26" s="2" t="n"/>
       <c r="P26" s="2" t="n"/>
-      <c r="Q26" s="2" t="n"/>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>developed country</t>
+        </is>
+      </c>
       <c r="R26" s="2" t="n"/>
-      <c r="S26" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T26" s="2" t="n"/>
+      <c r="S26" s="2" t="n"/>
+      <c r="T26" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U26" s="2" t="n"/>
-      <c r="V26" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V26" s="2" t="n"/>
       <c r="W26" s="2" t="inlineStr">
         <is>
-          <t>developed country</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X26" s="2" t="n"/>
@@ -2037,7 +2037,11 @@
           <t>A residential facility where an individual is living that is not stable and secure.</t>
         </is>
       </c>
-      <c r="D27" s="2" t="n"/>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>residential facility [OMRSE:00000191]</t>
+        </is>
+      </c>
       <c r="E27" s="2" t="n"/>
       <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="n"/>
@@ -2046,31 +2050,27 @@
       <c r="J27" s="2" t="n"/>
       <c r="K27" s="2" t="n"/>
       <c r="L27" s="2" t="n"/>
-      <c r="M27" s="2" t="inlineStr">
-        <is>
-          <t>residential facility [OMRSE:00000191]</t>
-        </is>
-      </c>
+      <c r="M27" s="2" t="n"/>
       <c r="N27" s="2" t="n"/>
       <c r="O27" s="2" t="n"/>
       <c r="P27" s="2" t="n"/>
-      <c r="Q27" s="2" t="n"/>
+      <c r="Q27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">an architectural structure for which an individual does not have a legal right to stay </t>
+        </is>
+      </c>
       <c r="R27" s="2" t="n"/>
-      <c r="S27" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T27" s="2" t="n"/>
+      <c r="S27" s="2" t="n"/>
+      <c r="T27" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U27" s="2" t="n"/>
-      <c r="V27" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V27" s="2" t="n"/>
       <c r="W27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">an architectural structure for which an individual does not have a legal right to stay </t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X27" s="2" t="n"/>
@@ -2100,7 +2100,7 @@
           <t>A health care facility that bears a function to provide healthcare to the sick or terminally ill</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>healthcare facility [OMRSE:00000102]</t>
         </is>
@@ -2115,14 +2115,14 @@
           <t>OMRSE:00000104</t>
         </is>
       </c>
-      <c r="S28" t="inlineStr">
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>Setting</t>
         </is>
       </c>
       <c r="AB28" t="inlineStr">
@@ -2147,7 +2147,7 @@
           <t>A facility that is run by a hospital organization, such as emergency departments, outpatient clinics and rehabilitation and is the bearer of a hospital function</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>healthcare facility [OMRSE:00000102]</t>
         </is>
@@ -2162,14 +2162,14 @@
           <t>OMRSE:00000063</t>
         </is>
       </c>
-      <c r="S29" t="inlineStr">
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="V29" t="inlineStr">
-        <is>
-          <t>Setting</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -2194,7 +2194,11 @@
           <t xml:space="preserve">A hospital facility to treat patients without them staying overnight, often after a hospital visit. </t>
         </is>
       </c>
-      <c r="D30" s="2" t="n"/>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>hospital facility [OMRSE:00000063]</t>
+        </is>
+      </c>
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="n"/>
@@ -2203,29 +2207,25 @@
       <c r="J30" s="2" t="n"/>
       <c r="K30" s="2" t="n"/>
       <c r="L30" s="2" t="n"/>
-      <c r="M30" s="2" t="inlineStr">
-        <is>
-          <t>hospital facility [OMRSE:00000063]</t>
-        </is>
-      </c>
+      <c r="M30" s="2" t="n"/>
       <c r="N30" s="2" t="n"/>
       <c r="O30" s="2" t="n"/>
       <c r="P30" s="2" t="n"/>
       <c r="Q30" s="2" t="n"/>
       <c r="R30" s="2" t="n"/>
-      <c r="S30" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T30" s="2" t="n"/>
+      <c r="S30" s="2" t="n"/>
+      <c r="T30" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U30" s="2" t="n"/>
-      <c r="V30" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W30" s="2" t="n"/>
+      <c r="V30" s="2" t="n"/>
+      <c r="W30" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X30" s="2" t="n"/>
       <c r="Y30" s="2" t="n"/>
       <c r="Z30" s="2" t="n"/>
@@ -2253,7 +2253,11 @@
           <t>A community facility used to serve food.</t>
         </is>
       </c>
-      <c r="D31" s="2" t="n"/>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>community facility [BCIO:026029]</t>
+        </is>
+      </c>
       <c r="E31" s="2" t="n"/>
       <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="n"/>
@@ -2262,31 +2266,27 @@
       <c r="J31" s="2" t="n"/>
       <c r="K31" s="2" t="n"/>
       <c r="L31" s="2" t="n"/>
-      <c r="M31" s="2" t="inlineStr">
-        <is>
-          <t>community facility [BCIO:026029]</t>
-        </is>
-      </c>
+      <c r="M31" s="2" t="n"/>
       <c r="N31" s="2" t="n"/>
       <c r="O31" s="2" t="n"/>
       <c r="P31" s="2" t="n"/>
-      <c r="Q31" s="2" t="n"/>
+      <c r="Q31" s="2" t="inlineStr">
+        <is>
+          <t>diner; restaurant; pub; bar</t>
+        </is>
+      </c>
       <c r="R31" s="2" t="n"/>
-      <c r="S31" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T31" s="2" t="n"/>
+      <c r="S31" s="2" t="n"/>
+      <c r="T31" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U31" s="2" t="n"/>
-      <c r="V31" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V31" s="2" t="n"/>
       <c r="W31" s="2" t="inlineStr">
         <is>
-          <t>diner; restaurant; pub; bar</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X31" s="2" t="n"/>
@@ -2316,7 +2316,11 @@
           <t>A facility where an individual is living alone or with one or more person. The individuals do not have to be related.</t>
         </is>
       </c>
-      <c r="D32" s="2" t="n"/>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>residential facility [OMRSE:00000191]</t>
+        </is>
+      </c>
       <c r="E32" s="2" t="n"/>
       <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="n"/>
@@ -2325,29 +2329,25 @@
       <c r="J32" s="2" t="n"/>
       <c r="K32" s="2" t="n"/>
       <c r="L32" s="2" t="n"/>
-      <c r="M32" s="2" t="inlineStr">
-        <is>
-          <t>residential facility [OMRSE:00000191]</t>
-        </is>
-      </c>
+      <c r="M32" s="2" t="n"/>
       <c r="N32" s="2" t="n"/>
       <c r="O32" s="2" t="n"/>
       <c r="P32" s="2" t="n"/>
       <c r="Q32" s="2" t="n"/>
       <c r="R32" s="2" t="n"/>
-      <c r="S32" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T32" s="2" t="n"/>
+      <c r="S32" s="2" t="n"/>
+      <c r="T32" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U32" s="2" t="n"/>
-      <c r="V32" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W32" s="2" t="n"/>
+      <c r="V32" s="2" t="n"/>
+      <c r="W32" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X32" s="2" t="n"/>
       <c r="Y32" s="2" t="n"/>
       <c r="Z32" s="2" t="n"/>
@@ -2375,7 +2375,11 @@
           <t>A community facility containing a collection of books and learning resources for loan.</t>
         </is>
       </c>
-      <c r="D33" s="2" t="n"/>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>community facility [BCIO:026029]</t>
+        </is>
+      </c>
       <c r="E33" s="2" t="n"/>
       <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="n"/>
@@ -2384,29 +2388,25 @@
       <c r="J33" s="2" t="n"/>
       <c r="K33" s="2" t="n"/>
       <c r="L33" s="2" t="n"/>
-      <c r="M33" s="2" t="inlineStr">
-        <is>
-          <t>community facility [BCIO:026029]</t>
-        </is>
-      </c>
+      <c r="M33" s="2" t="n"/>
       <c r="N33" s="2" t="n"/>
       <c r="O33" s="2" t="n"/>
       <c r="P33" s="2" t="n"/>
       <c r="Q33" s="2" t="n"/>
       <c r="R33" s="2" t="n"/>
-      <c r="S33" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T33" s="2" t="n"/>
+      <c r="S33" s="2" t="n"/>
+      <c r="T33" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U33" s="2" t="n"/>
-      <c r="V33" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W33" s="2" t="n"/>
+      <c r="V33" s="2" t="n"/>
+      <c r="W33" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X33" s="2" t="n"/>
       <c r="Y33" s="2" t="n"/>
       <c r="Z33" s="2" t="n"/>
@@ -2434,7 +2434,11 @@
           <t>An area social and economic condition described to have a low-income, whether at a country or within-country level.</t>
         </is>
       </c>
-      <c r="D34" s="2" t="n"/>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>area social and economic condition [BCIO:026004]</t>
+        </is>
+      </c>
       <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="n"/>
@@ -2443,29 +2447,25 @@
       <c r="J34" s="2" t="n"/>
       <c r="K34" s="2" t="n"/>
       <c r="L34" s="2" t="n"/>
-      <c r="M34" s="2" t="inlineStr">
-        <is>
-          <t>area social and economic condition [BCIO:026004]</t>
-        </is>
-      </c>
+      <c r="M34" s="2" t="n"/>
       <c r="N34" s="2" t="n"/>
       <c r="O34" s="2" t="n"/>
       <c r="P34" s="2" t="n"/>
       <c r="Q34" s="2" t="n"/>
       <c r="R34" s="2" t="n"/>
-      <c r="S34" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T34" s="2" t="n"/>
+      <c r="S34" s="2" t="n"/>
+      <c r="T34" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U34" s="2" t="n"/>
-      <c r="V34" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W34" s="2" t="n"/>
+      <c r="V34" s="2" t="n"/>
+      <c r="W34" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X34" s="2" t="n"/>
       <c r="Y34" s="2" t="n"/>
       <c r="Z34" s="2" t="n"/>
@@ -2493,7 +2493,11 @@
           <t>A school facility providing education between primary and secondary school.</t>
         </is>
       </c>
-      <c r="D35" s="2" t="n"/>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>school facility [OMRSE:00000064]</t>
+        </is>
+      </c>
       <c r="E35" s="2" t="n"/>
       <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="n"/>
@@ -2502,29 +2506,25 @@
       <c r="J35" s="2" t="n"/>
       <c r="K35" s="2" t="n"/>
       <c r="L35" s="2" t="n"/>
-      <c r="M35" s="2" t="inlineStr">
-        <is>
-          <t>school facility [OMRSE:00000064]</t>
-        </is>
-      </c>
+      <c r="M35" s="2" t="n"/>
       <c r="N35" s="2" t="n"/>
       <c r="O35" s="2" t="n"/>
       <c r="P35" s="2" t="n"/>
       <c r="Q35" s="2" t="n"/>
       <c r="R35" s="2" t="n"/>
-      <c r="S35" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T35" s="2" t="n"/>
+      <c r="S35" s="2" t="n"/>
+      <c r="T35" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U35" s="2" t="n"/>
-      <c r="V35" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W35" s="2" t="n"/>
+      <c r="V35" s="2" t="n"/>
+      <c r="W35" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X35" s="2" t="n"/>
       <c r="Y35" s="2" t="n"/>
       <c r="Z35" s="2" t="n"/>
@@ -2552,7 +2552,11 @@
           <t xml:space="preserve">A facility relating to or characteristic of soldiers or armed forces </t>
         </is>
       </c>
-      <c r="D36" s="2" t="n"/>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>facility [OMRSE:00000062]</t>
+        </is>
+      </c>
       <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="n"/>
@@ -2561,31 +2565,27 @@
       <c r="J36" s="2" t="n"/>
       <c r="K36" s="2" t="n"/>
       <c r="L36" s="2" t="n"/>
-      <c r="M36" s="2" t="inlineStr">
-        <is>
-          <t>facility [OMRSE:00000062]</t>
-        </is>
-      </c>
+      <c r="M36" s="2" t="n"/>
       <c r="N36" s="2" t="n"/>
       <c r="O36" s="2" t="n"/>
       <c r="P36" s="2" t="n"/>
-      <c r="Q36" s="2" t="n"/>
+      <c r="Q36" s="2" t="inlineStr">
+        <is>
+          <t>army; navy; air force</t>
+        </is>
+      </c>
       <c r="R36" s="2" t="n"/>
-      <c r="S36" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T36" s="2" t="n"/>
+      <c r="S36" s="2" t="n"/>
+      <c r="T36" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U36" s="2" t="n"/>
-      <c r="V36" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V36" s="2" t="n"/>
       <c r="W36" s="2" t="inlineStr">
         <is>
-          <t>army; navy; air force</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X36" s="2" t="n"/>
@@ -2615,7 +2615,11 @@
           <t>A form of transportation delivering interventions in transient locations.</t>
         </is>
       </c>
-      <c r="D37" s="2" t="n"/>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>transportation [BCIO:026041]</t>
+        </is>
+      </c>
       <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="n"/>
@@ -2624,31 +2628,27 @@
       <c r="J37" s="2" t="n"/>
       <c r="K37" s="2" t="n"/>
       <c r="L37" s="2" t="n"/>
-      <c r="M37" s="2" t="inlineStr">
-        <is>
-          <t>transportation [BCIO:026041]</t>
-        </is>
-      </c>
+      <c r="M37" s="2" t="n"/>
       <c r="N37" s="2" t="n"/>
       <c r="O37" s="2" t="n"/>
       <c r="P37" s="2" t="n"/>
-      <c r="Q37" s="2" t="n"/>
+      <c r="Q37" s="2" t="inlineStr">
+        <is>
+          <t>mobile van</t>
+        </is>
+      </c>
       <c r="R37" s="2" t="n"/>
-      <c r="S37" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T37" s="2" t="n"/>
+      <c r="S37" s="2" t="n"/>
+      <c r="T37" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U37" s="2" t="n"/>
-      <c r="V37" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V37" s="2" t="n"/>
       <c r="W37" s="2" t="inlineStr">
         <is>
-          <t>mobile van</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X37" s="2" t="n"/>
@@ -2678,7 +2678,11 @@
           <t>A facility where an individual lives with many others that may be collected according to a social structure such as education or disability.</t>
         </is>
       </c>
-      <c r="D38" s="2" t="n"/>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>residential facility [OMRSE:00000191]</t>
+        </is>
+      </c>
       <c r="E38" s="2" t="n"/>
       <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="n"/>
@@ -2687,31 +2691,27 @@
       <c r="J38" s="2" t="n"/>
       <c r="K38" s="2" t="n"/>
       <c r="L38" s="2" t="n"/>
-      <c r="M38" s="2" t="inlineStr">
-        <is>
-          <t>residential facility [OMRSE:00000191]</t>
-        </is>
-      </c>
+      <c r="M38" s="2" t="n"/>
       <c r="N38" s="2" t="n"/>
       <c r="O38" s="2" t="n"/>
       <c r="P38" s="2" t="n"/>
-      <c r="Q38" s="2" t="n"/>
+      <c r="Q38" s="2" t="inlineStr">
+        <is>
+          <t>bedsit</t>
+        </is>
+      </c>
       <c r="R38" s="2" t="n"/>
-      <c r="S38" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T38" s="2" t="n"/>
+      <c r="S38" s="2" t="n"/>
+      <c r="T38" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U38" s="2" t="n"/>
-      <c r="V38" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V38" s="2" t="n"/>
       <c r="W38" s="2" t="inlineStr">
         <is>
-          <t>bedsit</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X38" s="2" t="n"/>
@@ -2741,7 +2741,11 @@
           <t>A facility of a room, set of rooms, or building used as a place for commercial, professional, or bureaucratic work.</t>
         </is>
       </c>
-      <c r="D39" s="2" t="n"/>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>facility [OMRSE:00000062]</t>
+        </is>
+      </c>
       <c r="E39" s="2" t="n"/>
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="n"/>
@@ -2750,29 +2754,25 @@
       <c r="J39" s="2" t="n"/>
       <c r="K39" s="2" t="n"/>
       <c r="L39" s="2" t="n"/>
-      <c r="M39" s="2" t="inlineStr">
-        <is>
-          <t>facility [OMRSE:00000062]</t>
-        </is>
-      </c>
+      <c r="M39" s="2" t="n"/>
       <c r="N39" s="2" t="n"/>
       <c r="O39" s="2" t="n"/>
       <c r="P39" s="2" t="n"/>
       <c r="Q39" s="2" t="n"/>
       <c r="R39" s="2" t="n"/>
-      <c r="S39" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T39" s="2" t="n"/>
+      <c r="S39" s="2" t="n"/>
+      <c r="T39" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U39" s="2" t="n"/>
-      <c r="V39" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W39" s="2" t="n"/>
+      <c r="V39" s="2" t="n"/>
+      <c r="W39" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X39" s="2" t="n"/>
       <c r="Y39" s="2" t="n"/>
       <c r="Z39" s="2" t="n"/>
@@ -2800,7 +2800,11 @@
           <t xml:space="preserve">A site which is an outdoor location outside of a building. </t>
         </is>
       </c>
-      <c r="D40" s="2" t="n"/>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>site [BFO:0000029]</t>
+        </is>
+      </c>
       <c r="E40" s="2" t="n"/>
       <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="n"/>
@@ -2809,29 +2813,25 @@
       <c r="J40" s="2" t="n"/>
       <c r="K40" s="2" t="n"/>
       <c r="L40" s="2" t="n"/>
-      <c r="M40" s="2" t="inlineStr">
-        <is>
-          <t>site [BFO:0000029]</t>
-        </is>
-      </c>
+      <c r="M40" s="2" t="n"/>
       <c r="N40" s="2" t="n"/>
       <c r="O40" s="2" t="n"/>
       <c r="P40" s="2" t="n"/>
       <c r="Q40" s="2" t="n"/>
       <c r="R40" s="2" t="n"/>
-      <c r="S40" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T40" s="2" t="n"/>
+      <c r="S40" s="2" t="n"/>
+      <c r="T40" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U40" s="2" t="n"/>
-      <c r="V40" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W40" s="2" t="n"/>
+      <c r="V40" s="2" t="n"/>
+      <c r="W40" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X40" s="2" t="n"/>
       <c r="Y40" s="2" t="n"/>
       <c r="Z40" s="2" t="n"/>
@@ -2859,7 +2859,7 @@
           <t>A bounded area of land, or water, usually in its natural or semi-natural (landscaped) state and set aside for some purpose, usually to do with recreation or conservation</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>outdoor environment [BCIO:026046]</t>
         </is>
@@ -2874,14 +2874,14 @@
           <t>ENVO:00000562</t>
         </is>
       </c>
-      <c r="S41" t="inlineStr">
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="V41" t="inlineStr">
-        <is>
-          <t>Setting</t>
         </is>
       </c>
       <c r="AB41" t="inlineStr">
@@ -2906,7 +2906,11 @@
           <t>An outdoor environment for the passage of persons or cyclists on land</t>
         </is>
       </c>
-      <c r="D42" s="2" t="n"/>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>outdoor environment [BCIO:026046]</t>
+        </is>
+      </c>
       <c r="E42" s="2" t="n"/>
       <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="n"/>
@@ -2915,29 +2919,25 @@
       <c r="J42" s="2" t="n"/>
       <c r="K42" s="2" t="n"/>
       <c r="L42" s="2" t="n"/>
-      <c r="M42" s="2" t="inlineStr">
-        <is>
-          <t>outdoor environment [BCIO:026046]</t>
-        </is>
-      </c>
+      <c r="M42" s="2" t="n"/>
       <c r="N42" s="2" t="n"/>
       <c r="O42" s="2" t="n"/>
       <c r="P42" s="2" t="n"/>
       <c r="Q42" s="2" t="n"/>
       <c r="R42" s="2" t="n"/>
-      <c r="S42" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T42" s="2" t="n"/>
+      <c r="S42" s="2" t="n"/>
+      <c r="T42" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U42" s="2" t="n"/>
-      <c r="V42" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W42" s="2" t="n"/>
+      <c r="V42" s="2" t="n"/>
+      <c r="W42" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X42" s="2" t="n"/>
       <c r="Y42" s="2" t="n"/>
       <c r="Z42" s="2" t="n"/>
@@ -2965,7 +2965,11 @@
           <t>A path or pavement for the passage of people using bicycles only on land.</t>
         </is>
       </c>
-      <c r="D43" s="2" t="n"/>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>path or pavement [BCIO:026048]</t>
+        </is>
+      </c>
       <c r="E43" s="2" t="n"/>
       <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="n"/>
@@ -2974,29 +2978,25 @@
       <c r="J43" s="2" t="n"/>
       <c r="K43" s="2" t="n"/>
       <c r="L43" s="2" t="n"/>
-      <c r="M43" s="2" t="inlineStr">
-        <is>
-          <t>path or pavement [BCIO:026048]</t>
-        </is>
-      </c>
+      <c r="M43" s="2" t="n"/>
       <c r="N43" s="2" t="n"/>
       <c r="O43" s="2" t="n"/>
       <c r="P43" s="2" t="n"/>
       <c r="Q43" s="2" t="n"/>
       <c r="R43" s="2" t="n"/>
-      <c r="S43" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T43" s="2" t="n"/>
+      <c r="S43" s="2" t="n"/>
+      <c r="T43" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U43" s="2" t="n"/>
-      <c r="V43" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W43" s="2" t="n"/>
+      <c r="V43" s="2" t="n"/>
+      <c r="W43" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X43" s="2" t="n"/>
       <c r="Y43" s="2" t="n"/>
       <c r="Z43" s="2" t="n"/>
@@ -3024,7 +3024,11 @@
           <t>A path or pavement for the passage of persons only on land.</t>
         </is>
       </c>
-      <c r="D44" s="2" t="n"/>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>path or pavement [BCIO:026048]</t>
+        </is>
+      </c>
       <c r="E44" s="2" t="n"/>
       <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="n"/>
@@ -3033,29 +3037,25 @@
       <c r="J44" s="2" t="n"/>
       <c r="K44" s="2" t="n"/>
       <c r="L44" s="2" t="n"/>
-      <c r="M44" s="2" t="inlineStr">
-        <is>
-          <t>path or pavement [BCIO:026048]</t>
-        </is>
-      </c>
+      <c r="M44" s="2" t="n"/>
       <c r="N44" s="2" t="n"/>
       <c r="O44" s="2" t="n"/>
       <c r="P44" s="2" t="n"/>
       <c r="Q44" s="2" t="n"/>
       <c r="R44" s="2" t="n"/>
-      <c r="S44" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T44" s="2" t="n"/>
+      <c r="S44" s="2" t="n"/>
+      <c r="T44" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U44" s="2" t="n"/>
-      <c r="V44" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W44" s="2" t="n"/>
+      <c r="V44" s="2" t="n"/>
+      <c r="W44" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X44" s="2" t="n"/>
       <c r="Y44" s="2" t="n"/>
       <c r="Z44" s="2" t="n"/>
@@ -3083,7 +3083,7 @@
           <t>A health care facility whose function is to store, prepare, dispense, and monitor the usage of pharmaceutical drugs among patients in a given area or encountered in a given health care provider organization</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>healthcare facility [OMRSE:00000102]</t>
         </is>
@@ -3098,14 +3098,14 @@
           <t>PDRO:0000074</t>
         </is>
       </c>
-      <c r="S45" t="inlineStr">
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="V45" t="inlineStr">
-        <is>
-          <t>Setting</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -3130,7 +3130,11 @@
           <t>An attribute of location describing the density of an area, in terms of people and resources within it.</t>
         </is>
       </c>
-      <c r="D46" s="2" t="n"/>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>attribute of location [BCIO:026003]</t>
+        </is>
+      </c>
       <c r="E46" s="2" t="n"/>
       <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="n"/>
@@ -3139,29 +3143,25 @@
       <c r="J46" s="2" t="n"/>
       <c r="K46" s="2" t="n"/>
       <c r="L46" s="2" t="n"/>
-      <c r="M46" s="2" t="inlineStr">
-        <is>
-          <t>attribute of location [BCIO:026003]</t>
-        </is>
-      </c>
+      <c r="M46" s="2" t="n"/>
       <c r="N46" s="2" t="n"/>
       <c r="O46" s="2" t="n"/>
       <c r="P46" s="2" t="n"/>
       <c r="Q46" s="2" t="n"/>
       <c r="R46" s="2" t="n"/>
-      <c r="S46" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T46" s="2" t="n"/>
+      <c r="S46" s="2" t="n"/>
+      <c r="T46" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U46" s="2" t="n"/>
-      <c r="V46" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W46" s="2" t="n"/>
+      <c r="V46" s="2" t="n"/>
+      <c r="W46" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X46" s="2" t="n"/>
       <c r="Y46" s="2" t="n"/>
       <c r="Z46" s="2" t="n"/>
@@ -3189,7 +3189,11 @@
           <t>A school facility for younger children, typically aged between five and eleven.</t>
         </is>
       </c>
-      <c r="D47" s="2" t="n"/>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>school facility [OMRSE:00000064]</t>
+        </is>
+      </c>
       <c r="E47" s="2" t="n"/>
       <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="n"/>
@@ -3198,29 +3202,25 @@
       <c r="J47" s="2" t="n"/>
       <c r="K47" s="2" t="n"/>
       <c r="L47" s="2" t="n"/>
-      <c r="M47" s="2" t="inlineStr">
-        <is>
-          <t>school facility [OMRSE:00000064]</t>
-        </is>
-      </c>
+      <c r="M47" s="2" t="n"/>
       <c r="N47" s="2" t="n"/>
       <c r="O47" s="2" t="n"/>
       <c r="P47" s="2" t="n"/>
       <c r="Q47" s="2" t="n"/>
       <c r="R47" s="2" t="n"/>
-      <c r="S47" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T47" s="2" t="n"/>
+      <c r="S47" s="2" t="n"/>
+      <c r="T47" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U47" s="2" t="n"/>
-      <c r="V47" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W47" s="2" t="n"/>
+      <c r="V47" s="2" t="n"/>
+      <c r="W47" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X47" s="2" t="n"/>
       <c r="Y47" s="2" t="n"/>
       <c r="Z47" s="2" t="n"/>
@@ -3248,7 +3248,11 @@
           <t>A form of transportation owned by an individual for individual or group use.</t>
         </is>
       </c>
-      <c r="D48" s="2" t="n"/>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>transportation [BCIO:026041]</t>
+        </is>
+      </c>
       <c r="E48" s="2" t="n"/>
       <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="n"/>
@@ -3257,31 +3261,27 @@
       <c r="J48" s="2" t="n"/>
       <c r="K48" s="2" t="n"/>
       <c r="L48" s="2" t="n"/>
-      <c r="M48" s="2" t="inlineStr">
-        <is>
-          <t>transportation [BCIO:026041]</t>
-        </is>
-      </c>
+      <c r="M48" s="2" t="n"/>
       <c r="N48" s="2" t="n"/>
       <c r="O48" s="2" t="n"/>
       <c r="P48" s="2" t="n"/>
-      <c r="Q48" s="2" t="n"/>
+      <c r="Q48" s="2" t="inlineStr">
+        <is>
+          <t>car; bicycle; motorbike</t>
+        </is>
+      </c>
       <c r="R48" s="2" t="n"/>
-      <c r="S48" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T48" s="2" t="n"/>
+      <c r="S48" s="2" t="n"/>
+      <c r="T48" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U48" s="2" t="n"/>
-      <c r="V48" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V48" s="2" t="n"/>
       <c r="W48" s="2" t="inlineStr">
         <is>
-          <t>car; bicycle; motorbike</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X48" s="2" t="n"/>
@@ -3311,7 +3311,11 @@
           <t>A place designed and staffed to house and treat individuals that need assistance with mental dysfunctions</t>
         </is>
       </c>
-      <c r="D49" s="2" t="n"/>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>healthcare facility [OMRSE:00000102]</t>
+        </is>
+      </c>
       <c r="E49" s="2" t="n"/>
       <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="n"/>
@@ -3320,11 +3324,7 @@
       <c r="J49" s="2" t="n"/>
       <c r="K49" s="2" t="n"/>
       <c r="L49" s="2" t="n"/>
-      <c r="M49" s="2" t="inlineStr">
-        <is>
-          <t>healthcare facility [OMRSE:00000102]</t>
-        </is>
-      </c>
+      <c r="M49" s="2" t="n"/>
       <c r="N49" s="2" t="n"/>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3338,19 +3338,19 @@
           <t>NCIT:C53536</t>
         </is>
       </c>
-      <c r="S49" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T49" s="2" t="n"/>
+      <c r="S49" s="2" t="n"/>
+      <c r="T49" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U49" s="2" t="n"/>
-      <c r="V49" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W49" s="2" t="n"/>
+      <c r="V49" s="2" t="n"/>
+      <c r="W49" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X49" s="2" t="n"/>
       <c r="Y49" s="2" t="n"/>
       <c r="Z49" s="2" t="n"/>
@@ -3378,7 +3378,11 @@
           <t>Forms of transportation that run on fixed routes and are available to the public, usually for a set fare</t>
         </is>
       </c>
-      <c r="D50" s="2" t="n"/>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>transportation [BCIO:026041]</t>
+        </is>
+      </c>
       <c r="E50" s="2" t="n"/>
       <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="n"/>
@@ -3387,11 +3391,7 @@
       <c r="J50" s="2" t="n"/>
       <c r="K50" s="2" t="n"/>
       <c r="L50" s="2" t="n"/>
-      <c r="M50" s="2" t="inlineStr">
-        <is>
-          <t>transportation [BCIO:026041]</t>
-        </is>
-      </c>
+      <c r="M50" s="2" t="n"/>
       <c r="N50" s="2" t="n"/>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3399,27 +3399,27 @@
         </is>
       </c>
       <c r="P50" s="2" t="n"/>
-      <c r="Q50" s="2" t="n"/>
+      <c r="Q50" s="2" t="inlineStr">
+        <is>
+          <t>bus; train; plane</t>
+        </is>
+      </c>
       <c r="R50" s="2" t="inlineStr">
         <is>
           <t>NCIT:C141287</t>
         </is>
       </c>
-      <c r="S50" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T50" s="2" t="n"/>
+      <c r="S50" s="2" t="n"/>
+      <c r="T50" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U50" s="2" t="n"/>
-      <c r="V50" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V50" s="2" t="n"/>
       <c r="W50" s="2" t="inlineStr">
         <is>
-          <t>bus; train; plane</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X50" s="2" t="n"/>
@@ -3449,7 +3449,7 @@
           <t>A facility to assist in physical or addiction recovery</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>healthcare facility [OMRSE:00000102]</t>
         </is>
@@ -3464,14 +3464,14 @@
           <t>OMRSE:00000106</t>
         </is>
       </c>
-      <c r="S51" t="inlineStr">
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="V51" t="inlineStr">
-        <is>
-          <t>Setting</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -3496,7 +3496,11 @@
           <t>A community facility where individuals or a group of people come to perform acts of devotion and veneration.</t>
         </is>
       </c>
-      <c r="D52" s="2" t="n"/>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>community facility [BCIO:026029]</t>
+        </is>
+      </c>
       <c r="E52" s="2" t="n"/>
       <c r="F52" s="2" t="n"/>
       <c r="G52" s="2" t="n"/>
@@ -3505,31 +3509,27 @@
       <c r="J52" s="2" t="n"/>
       <c r="K52" s="2" t="n"/>
       <c r="L52" s="2" t="n"/>
-      <c r="M52" s="2" t="inlineStr">
-        <is>
-          <t>community facility [BCIO:026029]</t>
-        </is>
-      </c>
+      <c r="M52" s="2" t="n"/>
       <c r="N52" s="2" t="n"/>
       <c r="O52" s="2" t="n"/>
       <c r="P52" s="2" t="n"/>
-      <c r="Q52" s="2" t="n"/>
+      <c r="Q52" s="2" t="inlineStr">
+        <is>
+          <t>mosque; church; temple</t>
+        </is>
+      </c>
       <c r="R52" s="2" t="n"/>
-      <c r="S52" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T52" s="2" t="n"/>
+      <c r="S52" s="2" t="n"/>
+      <c r="T52" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U52" s="2" t="n"/>
-      <c r="V52" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V52" s="2" t="n"/>
       <c r="W52" s="2" t="inlineStr">
         <is>
-          <t>mosque; church; temple</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X52" s="2" t="n"/>
@@ -3559,7 +3559,7 @@
           <t>A facility, permanent or temporary, on land, in air, space or water, where scientific research or measurements can be undertaken</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>facility [OMRSE:00000062]</t>
         </is>
@@ -3569,24 +3569,24 @@
           <t>Environment Ontology</t>
         </is>
       </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>research lab</t>
+        </is>
+      </c>
       <c r="R53" t="inlineStr">
         <is>
           <t>ENVO:00000469</t>
         </is>
       </c>
-      <c r="S53" t="inlineStr">
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="W53" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="V53" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W53" t="inlineStr">
-        <is>
-          <t>research lab</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -3611,7 +3611,11 @@
           <t>A multiple occupancy residence where multiple vulnerable people live</t>
         </is>
       </c>
-      <c r="D54" s="2" t="n"/>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>multiple occupancy residence [BCIO:026010]</t>
+        </is>
+      </c>
       <c r="E54" s="2" t="n"/>
       <c r="F54" s="2" t="n"/>
       <c r="G54" s="2" t="n"/>
@@ -3620,31 +3624,27 @@
       <c r="J54" s="2" t="n"/>
       <c r="K54" s="2" t="n"/>
       <c r="L54" s="2" t="n"/>
-      <c r="M54" s="2" t="inlineStr">
-        <is>
-          <t>multiple occupancy residence [BCIO:026010]</t>
-        </is>
-      </c>
+      <c r="M54" s="2" t="n"/>
       <c r="N54" s="2" t="n"/>
       <c r="O54" s="2" t="n"/>
       <c r="P54" s="2" t="n"/>
-      <c r="Q54" s="2" t="n"/>
+      <c r="Q54" s="2" t="inlineStr">
+        <is>
+          <t>retirement home</t>
+        </is>
+      </c>
       <c r="R54" s="2" t="n"/>
-      <c r="S54" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T54" s="2" t="n"/>
+      <c r="S54" s="2" t="n"/>
+      <c r="T54" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U54" s="2" t="n"/>
-      <c r="V54" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V54" s="2" t="n"/>
       <c r="W54" s="2" t="inlineStr">
         <is>
-          <t>retirement home</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X54" s="2" t="n"/>
@@ -3674,7 +3674,7 @@
           <t>A facility that has at least one housing unit as part in which a person or persons live</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr">
+      <c r="D55" t="inlineStr">
         <is>
           <t>facility [OMRSE:00000062]</t>
         </is>
@@ -3689,14 +3689,14 @@
           <t>OMRSE:00000191</t>
         </is>
       </c>
-      <c r="S55" t="inlineStr">
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="W55" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="V55" t="inlineStr">
-        <is>
-          <t>Setting</t>
         </is>
       </c>
       <c r="AB55" t="inlineStr">
@@ -3721,7 +3721,11 @@
           <t>A facility used as an outlet for shopping.</t>
         </is>
       </c>
-      <c r="D56" s="2" t="n"/>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>facility [OMRSE:00000062]</t>
+        </is>
+      </c>
       <c r="E56" s="2" t="n"/>
       <c r="F56" s="2" t="n"/>
       <c r="G56" s="2" t="n"/>
@@ -3730,31 +3734,27 @@
       <c r="J56" s="2" t="n"/>
       <c r="K56" s="2" t="n"/>
       <c r="L56" s="2" t="n"/>
-      <c r="M56" s="2" t="inlineStr">
-        <is>
-          <t>facility [OMRSE:00000062]</t>
-        </is>
-      </c>
+      <c r="M56" s="2" t="n"/>
       <c r="N56" s="2" t="n"/>
       <c r="O56" s="2" t="n"/>
       <c r="P56" s="2" t="n"/>
-      <c r="Q56" s="2" t="n"/>
+      <c r="Q56" s="2" t="inlineStr">
+        <is>
+          <t>supermarket; market; shopping centre</t>
+        </is>
+      </c>
       <c r="R56" s="2" t="n"/>
-      <c r="S56" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T56" s="2" t="n"/>
+      <c r="S56" s="2" t="n"/>
+      <c r="T56" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U56" s="2" t="n"/>
-      <c r="V56" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V56" s="2" t="n"/>
       <c r="W56" s="2" t="inlineStr">
         <is>
-          <t>supermarket; market; shopping centre</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X56" s="2" t="n"/>
@@ -3784,7 +3784,7 @@
           <t>An open way for the passage of vehicles, persons, or animals on land</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr">
+      <c r="D57" t="inlineStr">
         <is>
           <t>outdoor environment [BCIO:026046]</t>
         </is>
@@ -3799,16 +3799,16 @@
           <t>ENVO:00000064</t>
         </is>
       </c>
-      <c r="S57" t="inlineStr">
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="W57" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="V57" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
       <c r="AB57" t="inlineStr">
         <is>
           <t>0</t>
@@ -3816,46 +3816,67 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>BCIO:050915</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>rural area density</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>A population and resource density that involves being outside of an urban or suburban area and has a low density of population and buildings.</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>population and resource density [BCIO:026007]</t>
         </is>
       </c>
-      <c r="S58" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="V58" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="AA58" t="inlineStr">
+      <c r="E58" s="2" t="n"/>
+      <c r="F58" s="2" t="n"/>
+      <c r="G58" s="2" t="n"/>
+      <c r="H58" s="2" t="n"/>
+      <c r="I58" s="2" t="n"/>
+      <c r="J58" s="2" t="n"/>
+      <c r="K58" s="2" t="n"/>
+      <c r="L58" s="2" t="n"/>
+      <c r="M58" s="2" t="n"/>
+      <c r="N58" s="2" t="n"/>
+      <c r="O58" s="2" t="n"/>
+      <c r="P58" s="2" t="n"/>
+      <c r="Q58" s="2" t="n"/>
+      <c r="R58" s="2" t="n"/>
+      <c r="S58" s="2" t="n"/>
+      <c r="T58" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="U58" s="2" t="n"/>
+      <c r="V58" s="2" t="inlineStr">
         <is>
           <t>RW</t>
         </is>
       </c>
-      <c r="AB58" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="W58" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="X58" s="2" t="n"/>
+      <c r="Y58" s="2" t="n"/>
+      <c r="Z58" s="2" t="n"/>
+      <c r="AA58" s="2" t="n"/>
+      <c r="AB58" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AC58" s="2" t="n"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3873,7 +3894,7 @@
           <t>A facility that is run by a school organization and is the bearer of a school function</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr">
+      <c r="D59" t="inlineStr">
         <is>
           <t>educational facility [BCIO:026022]</t>
         </is>
@@ -3888,14 +3909,14 @@
           <t xml:space="preserve">OMRSE:00000064 </t>
         </is>
       </c>
-      <c r="S59" t="inlineStr">
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="W59" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="V59" t="inlineStr">
-        <is>
-          <t>Setting</t>
         </is>
       </c>
       <c r="AB59" t="inlineStr">
@@ -3920,7 +3941,11 @@
           <t>A school facility for older children and teenagers, typically aged between eleven and eighteen.</t>
         </is>
       </c>
-      <c r="D60" s="2" t="n"/>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>school facility [OMRSE:00000064]</t>
+        </is>
+      </c>
       <c r="E60" s="2" t="n"/>
       <c r="F60" s="2" t="n"/>
       <c r="G60" s="2" t="n"/>
@@ -3929,31 +3954,27 @@
       <c r="J60" s="2" t="n"/>
       <c r="K60" s="2" t="n"/>
       <c r="L60" s="2" t="n"/>
-      <c r="M60" s="2" t="inlineStr">
-        <is>
-          <t>school facility [OMRSE:00000064]</t>
-        </is>
-      </c>
+      <c r="M60" s="2" t="n"/>
       <c r="N60" s="2" t="n"/>
       <c r="O60" s="2" t="n"/>
       <c r="P60" s="2" t="n"/>
-      <c r="Q60" s="2" t="n"/>
+      <c r="Q60" s="2" t="inlineStr">
+        <is>
+          <t>high school</t>
+        </is>
+      </c>
       <c r="R60" s="2" t="n"/>
-      <c r="S60" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T60" s="2" t="n"/>
+      <c r="S60" s="2" t="n"/>
+      <c r="T60" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U60" s="2" t="n"/>
-      <c r="V60" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V60" s="2" t="n"/>
       <c r="W60" s="2" t="inlineStr">
         <is>
-          <t>high school</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X60" s="2" t="n"/>
@@ -3983,7 +4004,7 @@
           <t>A three-dimensional immaterial entity that is (partially or wholly) bounded by a material entity or it is a three-dimensional immaterial part thereof.</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr">
+      <c r="D61" t="inlineStr">
         <is>
           <t>immaterial entity</t>
         </is>
@@ -3998,19 +4019,19 @@
           <t>BFO_0000029</t>
         </is>
       </c>
-      <c r="S61" t="inlineStr">
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="W61" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="V61" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="AA61" t="inlineStr">
-        <is>
-          <t>RW</t>
         </is>
       </c>
       <c r="AB61" t="inlineStr">
@@ -4035,7 +4056,11 @@
           <t>A community facility used for socialising by those living in a given area.</t>
         </is>
       </c>
-      <c r="D62" s="2" t="n"/>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>community facility [BCIO:026029]</t>
+        </is>
+      </c>
       <c r="E62" s="2" t="n"/>
       <c r="F62" s="2" t="n"/>
       <c r="G62" s="2" t="n"/>
@@ -4044,31 +4069,27 @@
       <c r="J62" s="2" t="n"/>
       <c r="K62" s="2" t="n"/>
       <c r="L62" s="2" t="n"/>
-      <c r="M62" s="2" t="inlineStr">
-        <is>
-          <t>community facility [BCIO:026029]</t>
-        </is>
-      </c>
+      <c r="M62" s="2" t="n"/>
       <c r="N62" s="2" t="n"/>
       <c r="O62" s="2" t="n"/>
       <c r="P62" s="2" t="n"/>
-      <c r="Q62" s="2" t="n"/>
+      <c r="Q62" s="2" t="inlineStr">
+        <is>
+          <t>YMCA; working mens club</t>
+        </is>
+      </c>
       <c r="R62" s="2" t="n"/>
-      <c r="S62" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T62" s="2" t="n"/>
+      <c r="S62" s="2" t="n"/>
+      <c r="T62" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U62" s="2" t="n"/>
-      <c r="V62" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V62" s="2" t="n"/>
       <c r="W62" s="2" t="inlineStr">
         <is>
-          <t>YMCA; working mens club</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X62" s="2" t="n"/>
@@ -4098,7 +4119,11 @@
           <t>A community facility used for exercising.</t>
         </is>
       </c>
-      <c r="D63" s="2" t="n"/>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>community facility [BCIO:026029]</t>
+        </is>
+      </c>
       <c r="E63" s="2" t="n"/>
       <c r="F63" s="2" t="n"/>
       <c r="G63" s="2" t="n"/>
@@ -4107,31 +4132,27 @@
       <c r="J63" s="2" t="n"/>
       <c r="K63" s="2" t="n"/>
       <c r="L63" s="2" t="n"/>
-      <c r="M63" s="2" t="inlineStr">
-        <is>
-          <t>community facility [BCIO:026029]</t>
-        </is>
-      </c>
+      <c r="M63" s="2" t="n"/>
       <c r="N63" s="2" t="n"/>
       <c r="O63" s="2" t="n"/>
       <c r="P63" s="2" t="n"/>
-      <c r="Q63" s="2" t="n"/>
+      <c r="Q63" s="2" t="inlineStr">
+        <is>
+          <t>gym; stadium; tennis court; swimming pool</t>
+        </is>
+      </c>
       <c r="R63" s="2" t="n"/>
-      <c r="S63" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T63" s="2" t="n"/>
+      <c r="S63" s="2" t="n"/>
+      <c r="T63" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U63" s="2" t="n"/>
-      <c r="V63" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V63" s="2" t="n"/>
       <c r="W63" s="2" t="inlineStr">
         <is>
-          <t>gym; stadium; tennis court; swimming pool</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X63" s="2" t="n"/>
@@ -4161,7 +4182,11 @@
           <t>A multiple occupancy residence where many students live.</t>
         </is>
       </c>
-      <c r="D64" s="2" t="n"/>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>multiple occupancy residence [BCIO:026010]</t>
+        </is>
+      </c>
       <c r="E64" s="2" t="n"/>
       <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="n"/>
@@ -4170,31 +4195,27 @@
       <c r="J64" s="2" t="n"/>
       <c r="K64" s="2" t="n"/>
       <c r="L64" s="2" t="n"/>
-      <c r="M64" s="2" t="inlineStr">
-        <is>
-          <t>multiple occupancy residence [BCIO:026010]</t>
-        </is>
-      </c>
+      <c r="M64" s="2" t="n"/>
       <c r="N64" s="2" t="n"/>
       <c r="O64" s="2" t="n"/>
       <c r="P64" s="2" t="n"/>
-      <c r="Q64" s="2" t="n"/>
+      <c r="Q64" s="2" t="inlineStr">
+        <is>
+          <t>student hall</t>
+        </is>
+      </c>
       <c r="R64" s="2" t="n"/>
-      <c r="S64" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T64" s="2" t="n"/>
+      <c r="S64" s="2" t="n"/>
+      <c r="T64" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U64" s="2" t="n"/>
-      <c r="V64" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V64" s="2" t="n"/>
       <c r="W64" s="2" t="inlineStr">
         <is>
-          <t>student hall</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X64" s="2" t="n"/>
@@ -4224,7 +4245,11 @@
           <t>A population and resource density that involves being on the edge of a large town or city where a proportion of those who work in the town or city live.</t>
         </is>
       </c>
-      <c r="D65" s="2" t="n"/>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>population and resource density [BCIO:026007]</t>
+        </is>
+      </c>
       <c r="E65" s="2" t="n"/>
       <c r="F65" s="2" t="n"/>
       <c r="G65" s="2" t="n"/>
@@ -4233,37 +4258,33 @@
       <c r="J65" s="2" t="n"/>
       <c r="K65" s="2" t="n"/>
       <c r="L65" s="2" t="n"/>
-      <c r="M65" s="2" t="inlineStr">
-        <is>
-          <t>population and resource density [BCIO:026007]</t>
-        </is>
-      </c>
+      <c r="M65" s="2" t="n"/>
       <c r="N65" s="2" t="n"/>
       <c r="O65" s="2" t="n"/>
       <c r="P65" s="2" t="n"/>
       <c r="Q65" s="2" t="n"/>
       <c r="R65" s="2" t="n"/>
-      <c r="S65" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T65" s="2" t="n"/>
+      <c r="S65" s="2" t="n"/>
+      <c r="T65" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U65" s="2" t="n"/>
       <c r="V65" s="2" t="inlineStr">
         <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W65" s="2" t="n"/>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="W65" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X65" s="2" t="n"/>
       <c r="Y65" s="2" t="n"/>
       <c r="Z65" s="2" t="n"/>
-      <c r="AA65" s="2" t="inlineStr">
-        <is>
-          <t>RW</t>
-        </is>
-      </c>
+      <c r="AA65" s="2" t="n"/>
       <c r="AB65" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -4287,7 +4308,11 @@
           <t xml:space="preserve">A residential facility where individuals are in a transitional state of housing and not staying for a prolonged period. </t>
         </is>
       </c>
-      <c r="D66" s="2" t="n"/>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>residential facility [OMRSE:00000191]</t>
+        </is>
+      </c>
       <c r="E66" s="2" t="n"/>
       <c r="F66" s="2" t="n"/>
       <c r="G66" s="2" t="n"/>
@@ -4296,31 +4321,27 @@
       <c r="J66" s="2" t="n"/>
       <c r="K66" s="2" t="n"/>
       <c r="L66" s="2" t="n"/>
-      <c r="M66" s="2" t="inlineStr">
-        <is>
-          <t>residential facility [OMRSE:00000191]</t>
-        </is>
-      </c>
+      <c r="M66" s="2" t="n"/>
       <c r="N66" s="2" t="n"/>
       <c r="O66" s="2" t="n"/>
       <c r="P66" s="2" t="n"/>
-      <c r="Q66" s="2" t="n"/>
+      <c r="Q66" s="2" t="inlineStr">
+        <is>
+          <t>Hostels; BandB; emergency accomnodation</t>
+        </is>
+      </c>
       <c r="R66" s="2" t="n"/>
-      <c r="S66" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T66" s="2" t="n"/>
+      <c r="S66" s="2" t="n"/>
+      <c r="T66" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U66" s="2" t="n"/>
-      <c r="V66" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
+      <c r="V66" s="2" t="n"/>
       <c r="W66" s="2" t="inlineStr">
         <is>
-          <t>Hostels; BandB; emergency accomnodation</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X66" s="2" t="n"/>
@@ -4350,7 +4371,11 @@
           <t>Methods of traveling from one place to another.</t>
         </is>
       </c>
-      <c r="D67" s="2" t="n"/>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>site [BFO:0000029]</t>
+        </is>
+      </c>
       <c r="E67" s="2" t="n"/>
       <c r="F67" s="2" t="n"/>
       <c r="G67" s="2" t="n"/>
@@ -4359,11 +4384,7 @@
       <c r="J67" s="2" t="n"/>
       <c r="K67" s="2" t="n"/>
       <c r="L67" s="2" t="n"/>
-      <c r="M67" s="2" t="inlineStr">
-        <is>
-          <t>site [BFO:0000029]</t>
-        </is>
-      </c>
+      <c r="M67" s="2" t="n"/>
       <c r="N67" s="2" t="n"/>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4377,19 +4398,19 @@
           <t>NCIT_C141286</t>
         </is>
       </c>
-      <c r="S67" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T67" s="2" t="n"/>
+      <c r="S67" s="2" t="n"/>
+      <c r="T67" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U67" s="2" t="n"/>
-      <c r="V67" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W67" s="2" t="n"/>
+      <c r="V67" s="2" t="n"/>
+      <c r="W67" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X67" s="2" t="n"/>
       <c r="Y67" s="2" t="n"/>
       <c r="Z67" s="2" t="n"/>
@@ -4417,7 +4438,11 @@
           <t>An educational facility in which students study for degrees and academic research is done.</t>
         </is>
       </c>
-      <c r="D68" s="2" t="n"/>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>educational facility [BCIO:026022]</t>
+        </is>
+      </c>
       <c r="E68" s="2" t="n"/>
       <c r="F68" s="2" t="n"/>
       <c r="G68" s="2" t="n"/>
@@ -4426,29 +4451,25 @@
       <c r="J68" s="2" t="n"/>
       <c r="K68" s="2" t="n"/>
       <c r="L68" s="2" t="n"/>
-      <c r="M68" s="2" t="inlineStr">
-        <is>
-          <t>educational facility [BCIO:026022]</t>
-        </is>
-      </c>
+      <c r="M68" s="2" t="n"/>
       <c r="N68" s="2" t="n"/>
       <c r="O68" s="2" t="n"/>
       <c r="P68" s="2" t="n"/>
       <c r="Q68" s="2" t="n"/>
       <c r="R68" s="2" t="n"/>
-      <c r="S68" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T68" s="2" t="n"/>
+      <c r="S68" s="2" t="n"/>
+      <c r="T68" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U68" s="2" t="n"/>
-      <c r="V68" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W68" s="2" t="n"/>
+      <c r="V68" s="2" t="n"/>
+      <c r="W68" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X68" s="2" t="n"/>
       <c r="Y68" s="2" t="n"/>
       <c r="Z68" s="2" t="n"/>
@@ -4461,51 +4482,71 @@
       <c r="AC68" s="2" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>BCIO:050914</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>urban area density</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
         <is>
           <t>A population and resource density that involves a high density of human population and of a built environment consisting of structures and infrastructure designed to support human habitation.</t>
         </is>
       </c>
-      <c r="M69" t="inlineStr">
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>population and resource density [BCIO:026007]</t>
         </is>
       </c>
-      <c r="O69" t="inlineStr">
+      <c r="E69" s="2" t="n"/>
+      <c r="F69" s="2" t="n"/>
+      <c r="G69" s="2" t="n"/>
+      <c r="H69" s="2" t="n"/>
+      <c r="I69" s="2" t="n"/>
+      <c r="J69" s="2" t="n"/>
+      <c r="K69" s="2" t="n"/>
+      <c r="L69" s="2" t="n"/>
+      <c r="M69" s="2" t="n"/>
+      <c r="N69" s="2" t="n"/>
+      <c r="O69" s="2" t="inlineStr">
         <is>
           <t>claude.ai</t>
         </is>
       </c>
-      <c r="S69" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="V69" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="AA69" t="inlineStr">
+      <c r="P69" s="2" t="n"/>
+      <c r="Q69" s="2" t="n"/>
+      <c r="R69" s="2" t="n"/>
+      <c r="S69" s="2" t="n"/>
+      <c r="T69" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="U69" s="2" t="n"/>
+      <c r="V69" s="2" t="inlineStr">
         <is>
           <t>RW</t>
         </is>
       </c>
-      <c r="AB69" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="W69" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="X69" s="2" t="n"/>
+      <c r="Y69" s="2" t="n"/>
+      <c r="Z69" s="2" t="n"/>
+      <c r="AA69" s="2" t="n"/>
+      <c r="AB69" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AC69" s="2" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4523,7 +4564,11 @@
           <t>An educational facility providing practically based, occupationally-specific teaching.</t>
         </is>
       </c>
-      <c r="D70" s="2" t="n"/>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>educational facility [BCIO:026022]</t>
+        </is>
+      </c>
       <c r="E70" s="2" t="n"/>
       <c r="F70" s="2" t="n"/>
       <c r="G70" s="2" t="n"/>
@@ -4532,29 +4577,25 @@
       <c r="J70" s="2" t="n"/>
       <c r="K70" s="2" t="n"/>
       <c r="L70" s="2" t="n"/>
-      <c r="M70" s="2" t="inlineStr">
-        <is>
-          <t>educational facility [BCIO:026022]</t>
-        </is>
-      </c>
+      <c r="M70" s="2" t="n"/>
       <c r="N70" s="2" t="n"/>
       <c r="O70" s="2" t="n"/>
       <c r="P70" s="2" t="n"/>
       <c r="Q70" s="2" t="n"/>
       <c r="R70" s="2" t="n"/>
-      <c r="S70" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T70" s="2" t="n"/>
+      <c r="S70" s="2" t="n"/>
+      <c r="T70" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U70" s="2" t="n"/>
-      <c r="V70" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W70" s="2" t="n"/>
+      <c r="V70" s="2" t="n"/>
+      <c r="W70" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X70" s="2" t="n"/>
       <c r="Y70" s="2" t="n"/>
       <c r="Z70" s="2" t="n"/>
@@ -4582,7 +4623,11 @@
           <t xml:space="preserve">An outdoor environment set in an expanse of water. </t>
         </is>
       </c>
-      <c r="D71" s="2" t="n"/>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>outdoor environment [BCIO:026046]</t>
+        </is>
+      </c>
       <c r="E71" s="2" t="n"/>
       <c r="F71" s="2" t="n"/>
       <c r="G71" s="2" t="n"/>
@@ -4591,29 +4636,25 @@
       <c r="J71" s="2" t="n"/>
       <c r="K71" s="2" t="n"/>
       <c r="L71" s="2" t="n"/>
-      <c r="M71" s="2" t="inlineStr">
-        <is>
-          <t>outdoor environment [BCIO:026046]</t>
-        </is>
-      </c>
+      <c r="M71" s="2" t="n"/>
       <c r="N71" s="2" t="n"/>
       <c r="O71" s="2" t="n"/>
       <c r="P71" s="2" t="n"/>
       <c r="Q71" s="2" t="n"/>
       <c r="R71" s="2" t="n"/>
-      <c r="S71" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T71" s="2" t="n"/>
+      <c r="S71" s="2" t="n"/>
+      <c r="T71" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U71" s="2" t="n"/>
-      <c r="V71" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="W71" s="2" t="n"/>
+      <c r="V71" s="2" t="n"/>
+      <c r="W71" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="X71" s="2" t="n"/>
       <c r="Y71" s="2" t="n"/>
       <c r="Z71" s="2" t="n"/>
@@ -4641,7 +4682,11 @@
           <t>A geographical location within a country.</t>
         </is>
       </c>
-      <c r="D72" s="2" t="n"/>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>geographic location [GAZ:00000448]</t>
+        </is>
+      </c>
       <c r="E72" s="2" t="n"/>
       <c r="F72" s="2" t="n"/>
       <c r="G72" s="2" t="n"/>
@@ -4650,41 +4695,37 @@
       <c r="J72" s="2" t="n"/>
       <c r="K72" s="2" t="n"/>
       <c r="L72" s="2" t="n"/>
-      <c r="M72" s="2" t="inlineStr">
-        <is>
-          <t>geographic location [GAZ:00000448]</t>
-        </is>
-      </c>
+      <c r="M72" s="2" t="n"/>
       <c r="N72" s="2" t="n"/>
       <c r="O72" s="2" t="n"/>
       <c r="P72" s="2" t="n"/>
-      <c r="Q72" s="2" t="n"/>
+      <c r="Q72" s="2" t="inlineStr">
+        <is>
+          <t>Region; Town; City; State; New York; Rotterdam</t>
+        </is>
+      </c>
       <c r="R72" s="2" t="n"/>
-      <c r="S72" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T72" s="2" t="n"/>
+      <c r="S72" s="2" t="n"/>
+      <c r="T72" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
       <c r="U72" s="2" t="n"/>
       <c r="V72" s="2" t="inlineStr">
         <is>
-          <t>Setting</t>
+          <t>LZ</t>
         </is>
       </c>
       <c r="W72" s="2" t="inlineStr">
         <is>
-          <t>Region; Town; City; State; New York; Rotterdam</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="X72" s="2" t="n"/>
       <c r="Y72" s="2" t="n"/>
       <c r="Z72" s="2" t="n"/>
-      <c r="AA72" s="2" t="inlineStr">
-        <is>
-          <t>LZ</t>
-        </is>
-      </c>
+      <c r="AA72" s="2" t="n"/>
       <c r="AB72" s="2" t="inlineStr">
         <is>
           <t>0</t>

</xml_diff>